<commit_message>
chore: baseline verificada antes del plan roles/eventos
</commit_message>
<xml_diff>
--- a/backend/data/profesores.xlsx
+++ b/backend/data/profesores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Axelgor\Documents\Programacion\proyectos\pisunpa-project\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D5B7974-128A-4D7E-83C6-3CA11395B81C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3AD647-CA98-4A9D-9F36-CF8941C40E43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D4CB3509-EC9A-4BCE-A9E2-4686A2604979}"/>
   </bookViews>
@@ -849,22 +849,58 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -878,42 +914,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1261,10 +1261,10 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="78" t="s">
+      <c r="A3" s="64" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="77" t="s">
+      <c r="B3" s="61" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="7"/>
@@ -1321,10 +1321,10 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="71" t="s">
+      <c r="A7" s="67" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="79" t="s">
+      <c r="B7" s="70" t="s">
         <v>15</v>
       </c>
       <c r="C7" s="15"/>
@@ -1339,8 +1339,8 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="72"/>
-      <c r="B8" s="80"/>
+      <c r="A8" s="68"/>
+      <c r="B8" s="71"/>
       <c r="C8" s="7"/>
       <c r="D8" s="1" t="s">
         <v>17</v>
@@ -1353,8 +1353,8 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="72"/>
-      <c r="B9" s="80"/>
+      <c r="A9" s="68"/>
+      <c r="B9" s="71"/>
       <c r="C9" s="7"/>
       <c r="D9" s="1" t="s">
         <v>17</v>
@@ -1367,8 +1367,8 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="73"/>
-      <c r="B10" s="81"/>
+      <c r="A10" s="69"/>
+      <c r="B10" s="72"/>
       <c r="C10" s="9"/>
       <c r="D10" s="10" t="s">
         <v>17</v>
@@ -1381,10 +1381,10 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="71" t="s">
+      <c r="A11" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="74" t="s">
+      <c r="B11" s="75" t="s">
         <v>22</v>
       </c>
       <c r="C11" s="14"/>
@@ -1399,8 +1399,8 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="72"/>
-      <c r="B12" s="75"/>
+      <c r="A12" s="68"/>
+      <c r="B12" s="76"/>
       <c r="C12" s="20"/>
       <c r="D12" s="21" t="s">
         <v>24</v>
@@ -1413,8 +1413,8 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="72"/>
-      <c r="B13" s="75"/>
+      <c r="A13" s="68"/>
+      <c r="B13" s="76"/>
       <c r="C13" s="20"/>
       <c r="D13" s="21" t="s">
         <v>24</v>
@@ -1427,8 +1427,8 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="73"/>
-      <c r="B14" s="76"/>
+      <c r="A14" s="69"/>
+      <c r="B14" s="77"/>
       <c r="C14" s="22"/>
       <c r="D14" s="23" t="s">
         <v>25</v>
@@ -1441,10 +1441,10 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="64" t="s">
+      <c r="A15" s="73" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="61" t="s">
+      <c r="B15" s="74" t="s">
         <v>30</v>
       </c>
       <c r="C15" s="15"/>
@@ -1489,10 +1489,10 @@
       <c r="F18" s="27"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="64" t="s">
+      <c r="A19" s="73" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="61" t="s">
+      <c r="B19" s="74" t="s">
         <v>35</v>
       </c>
       <c r="C19" s="15"/>
@@ -1541,10 +1541,10 @@
       <c r="F22" s="27"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="71" t="s">
+      <c r="A23" s="67" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="79" t="s">
+      <c r="B23" s="70" t="s">
         <v>41</v>
       </c>
       <c r="C23" s="15"/>
@@ -1559,8 +1559,8 @@
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="72"/>
-      <c r="B24" s="80"/>
+      <c r="A24" s="68"/>
+      <c r="B24" s="71"/>
       <c r="C24" s="7"/>
       <c r="D24" s="1" t="s">
         <v>42</v>
@@ -1573,8 +1573,8 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="72"/>
-      <c r="B25" s="80"/>
+      <c r="A25" s="68"/>
+      <c r="B25" s="71"/>
       <c r="C25" s="7"/>
       <c r="D25" s="1" t="s">
         <v>43</v>
@@ -1587,8 +1587,8 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="72"/>
-      <c r="B26" s="80"/>
+      <c r="A26" s="68"/>
+      <c r="B26" s="71"/>
       <c r="C26" s="7"/>
       <c r="D26" s="1" t="s">
         <v>43</v>
@@ -1601,8 +1601,8 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="72"/>
-      <c r="B27" s="80"/>
+      <c r="A27" s="68"/>
+      <c r="B27" s="71"/>
       <c r="C27" s="7"/>
       <c r="D27" s="1" t="s">
         <v>44</v>
@@ -1615,8 +1615,8 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="72"/>
-      <c r="B28" s="80"/>
+      <c r="A28" s="68"/>
+      <c r="B28" s="71"/>
       <c r="C28" s="7"/>
       <c r="D28" s="1" t="s">
         <v>45</v>
@@ -1629,8 +1629,8 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="73"/>
-      <c r="B29" s="81"/>
+      <c r="A29" s="69"/>
+      <c r="B29" s="72"/>
       <c r="C29" s="9"/>
       <c r="D29" s="10" t="s">
         <v>46</v>
@@ -1643,10 +1643,10 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="64" t="s">
+      <c r="A30" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="B30" s="61" t="s">
+      <c r="B30" s="74" t="s">
         <v>48</v>
       </c>
       <c r="C30" s="15"/>
@@ -1703,10 +1703,10 @@
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="64" t="s">
+      <c r="A34" s="73" t="s">
         <v>55</v>
       </c>
-      <c r="B34" s="61" t="s">
+      <c r="B34" s="74" t="s">
         <v>56</v>
       </c>
       <c r="C34" s="15"/>
@@ -1809,10 +1809,10 @@
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="64" t="s">
+      <c r="A41" s="73" t="s">
         <v>69</v>
       </c>
-      <c r="B41" s="82" t="s">
+      <c r="B41" s="78" t="s">
         <v>134</v>
       </c>
       <c r="C41" s="13"/>
@@ -1925,10 +1925,10 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="64" t="s">
+      <c r="A49" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="B49" s="82" t="s">
+      <c r="B49" s="78" t="s">
         <v>135</v>
       </c>
       <c r="C49" s="15"/>
@@ -1985,10 +1985,10 @@
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="64" t="s">
+      <c r="A53" s="73" t="s">
         <v>79</v>
       </c>
-      <c r="B53" s="61" t="s">
+      <c r="B53" s="74" t="s">
         <v>80</v>
       </c>
       <c r="C53" s="15"/>
@@ -2017,10 +2017,10 @@
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="64" t="s">
+      <c r="A55" s="73" t="s">
         <v>91</v>
       </c>
-      <c r="B55" s="61" t="s">
+      <c r="B55" s="74" t="s">
         <v>92</v>
       </c>
       <c r="C55" s="15"/>
@@ -2105,10 +2105,10 @@
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="64" t="s">
+      <c r="A61" s="73" t="s">
         <v>93</v>
       </c>
-      <c r="B61" s="61" t="s">
+      <c r="B61" s="74" t="s">
         <v>94</v>
       </c>
       <c r="C61" s="15"/>
@@ -2151,10 +2151,10 @@
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="64" t="s">
+      <c r="A64" s="73" t="s">
         <v>97</v>
       </c>
-      <c r="B64" s="61" t="s">
+      <c r="B64" s="74" t="s">
         <v>98</v>
       </c>
       <c r="C64" s="58"/>
@@ -2211,10 +2211,10 @@
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" s="67" t="s">
+      <c r="A68" s="79" t="s">
         <v>102</v>
       </c>
-      <c r="B68" s="69" t="s">
+      <c r="B68" s="81" t="s">
         <v>103</v>
       </c>
       <c r="C68" s="56"/>
@@ -2229,8 +2229,8 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" s="68"/>
-      <c r="B69" s="70"/>
+      <c r="A69" s="80"/>
+      <c r="B69" s="82"/>
       <c r="C69" s="57"/>
       <c r="D69" s="35" t="s">
         <v>104</v>
@@ -2243,10 +2243,10 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" s="64" t="s">
+      <c r="A70" s="73" t="s">
         <v>105</v>
       </c>
-      <c r="B70" s="61" t="s">
+      <c r="B70" s="74" t="s">
         <v>106</v>
       </c>
       <c r="C70" s="45"/>
@@ -2303,10 +2303,10 @@
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A74" s="64" t="s">
+      <c r="A74" s="73" t="s">
         <v>110</v>
       </c>
-      <c r="B74" s="82" t="s">
+      <c r="B74" s="78" t="s">
         <v>133</v>
       </c>
       <c r="C74" s="48"/>
@@ -2377,10 +2377,10 @@
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A79" s="64" t="s">
+      <c r="A79" s="73" t="s">
         <v>112</v>
       </c>
-      <c r="B79" s="61" t="s">
+      <c r="B79" s="74" t="s">
         <v>113</v>
       </c>
       <c r="C79" s="48"/>
@@ -2437,10 +2437,10 @@
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A83" s="64" t="s">
+      <c r="A83" s="73" t="s">
         <v>117</v>
       </c>
-      <c r="B83" s="61" t="s">
+      <c r="B83" s="74" t="s">
         <v>118</v>
       </c>
       <c r="C83" s="48"/>
@@ -2510,10 +2510,10 @@
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A88" s="64" t="s">
+      <c r="A88" s="73" t="s">
         <v>125</v>
       </c>
-      <c r="B88" s="61" t="s">
+      <c r="B88" s="74" t="s">
         <v>126</v>
       </c>
       <c r="C88" s="48"/>
@@ -2584,10 +2584,10 @@
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A93" s="64" t="s">
+      <c r="A93" s="73" t="s">
         <v>129</v>
       </c>
-      <c r="B93" s="61" t="s">
+      <c r="B93" s="74" t="s">
         <v>130</v>
       </c>
       <c r="C93" s="48"/>
@@ -2618,38 +2618,6 @@
   </sheetData>
   <autoFilter ref="A2:F94" xr:uid="{F6D26251-AA18-438C-A27A-01537EB07119}"/>
   <mergeCells count="42">
-    <mergeCell ref="B3:B6"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="A7:A10"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="B23:B29"/>
-    <mergeCell ref="A23:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="B11:B14"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="B15:B18"/>
-    <mergeCell ref="B19:B22"/>
-    <mergeCell ref="A19:A22"/>
-    <mergeCell ref="A34:A39"/>
-    <mergeCell ref="B34:B39"/>
-    <mergeCell ref="B41:B48"/>
-    <mergeCell ref="A41:A48"/>
-    <mergeCell ref="A49:A52"/>
-    <mergeCell ref="B49:B52"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="B55:B60"/>
-    <mergeCell ref="A55:A60"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="A61:A63"/>
-    <mergeCell ref="B64:B67"/>
-    <mergeCell ref="A64:A67"/>
-    <mergeCell ref="A68:A69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="A70:A73"/>
     <mergeCell ref="B88:B92"/>
     <mergeCell ref="A88:A92"/>
     <mergeCell ref="A93:A94"/>
@@ -2660,6 +2628,38 @@
     <mergeCell ref="A79:A82"/>
     <mergeCell ref="B83:B87"/>
     <mergeCell ref="A83:A87"/>
+    <mergeCell ref="B64:B67"/>
+    <mergeCell ref="A64:A67"/>
+    <mergeCell ref="A68:A69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="B55:B60"/>
+    <mergeCell ref="A55:A60"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="A61:A63"/>
+    <mergeCell ref="A34:A39"/>
+    <mergeCell ref="B34:B39"/>
+    <mergeCell ref="B41:B48"/>
+    <mergeCell ref="A41:A48"/>
+    <mergeCell ref="A49:A52"/>
+    <mergeCell ref="B49:B52"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="B11:B14"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="B15:B18"/>
+    <mergeCell ref="B19:B22"/>
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="B23:B29"/>
+    <mergeCell ref="A23:A29"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B74" r:id="rId1" xr:uid="{FC4BBA7A-A6CB-4E17-AD3D-76C23D0F39EF}"/>

</xml_diff>